<commit_message>
Add Sanity Categories column to spreadsheet and assign categories to all reviews
Added 'Sanity Categories' column with comma-separated category slugs for
all 29 reviewed tools. Each tool has 1-6 categories assigned based on
its functionality. Updated all Sanity documents with category references.

Categories mapped: project-management, task-management, team-collaboration,
workflow-automation, integration-platform, business-process-management,
database-software, no-code-platform, document-management, knowledge-management,
note-taking, time-tracking, marketing-automation, sales-automation.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content-templates/reviews/software_automation_tools.xlsx
+++ b/content-templates/reviews/software_automation_tools.xlsx
@@ -1425,7 +1425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L272"/>
+  <dimension ref="A1:M272"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1498,6 +1498,11 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Sanity Categories</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="12" t="inlineStr">
@@ -1563,6 +1568,11 @@
           <t>asana.md</t>
         </is>
       </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>project-management, task-management, team-collaboration</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
@@ -1615,6 +1625,11 @@
           <t>monday.md</t>
         </is>
       </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>project-management, task-management, team-collaboration, workflow-automation</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
@@ -1667,6 +1682,11 @@
           <t>jira.md</t>
         </is>
       </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>project-management, task-management, integration-platform</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
@@ -1719,6 +1739,11 @@
           <t>clickup.md</t>
         </is>
       </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>project-management, task-management, team-collaboration, document-management, time-tracking</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
@@ -1771,6 +1796,11 @@
           <t>trello.md</t>
         </is>
       </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>project-management, task-management, team-collaboration</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
@@ -1823,6 +1853,11 @@
           <t>basecamp.md</t>
         </is>
       </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>project-management, team-collaboration</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="inlineStr">
@@ -1875,6 +1910,11 @@
           <t>notion.md</t>
         </is>
       </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>project-management, knowledge-management, note-taking, team-collaboration, document-management, database-software</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -1927,6 +1967,11 @@
           <t>linear.md</t>
         </is>
       </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>project-management, task-management</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
@@ -2026,6 +2071,11 @@
           <t>wrike.md</t>
         </is>
       </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>project-management, task-management, team-collaboration, marketing-automation</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="inlineStr">
@@ -2078,6 +2128,11 @@
           <t>smartsheet.md</t>
         </is>
       </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>project-management, task-management, business-process-management</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
@@ -2130,6 +2185,11 @@
           <t>teamwork.md</t>
         </is>
       </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>project-management, task-management, time-tracking, team-collaboration</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="14" t="inlineStr">
@@ -2180,6 +2240,11 @@
       <c r="K15" t="inlineStr">
         <is>
           <t>airtable.md</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>project-management, database-software, no-code-platform, team-collaboration</t>
         </is>
       </c>
     </row>
@@ -3249,6 +3314,11 @@
           <t>zapier.md</t>
         </is>
       </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>workflow-automation, integration-platform, business-process-management</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="20" t="inlineStr">
@@ -3301,6 +3371,11 @@
           <t>make.md</t>
         </is>
       </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>workflow-automation, integration-platform, business-process-management</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="20" t="inlineStr">
@@ -3353,6 +3428,11 @@
           <t>n8n.md</t>
         </is>
       </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>workflow-automation, integration-platform, business-process-management</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="20" t="inlineStr">
@@ -3405,6 +3485,11 @@
           <t>pipedream.md</t>
         </is>
       </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>workflow-automation, integration-platform</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="20" t="inlineStr">
@@ -3457,6 +3542,11 @@
           <t>tray-io.md</t>
         </is>
       </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>workflow-automation, integration-platform, business-process-management</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="20" t="inlineStr">
@@ -3509,6 +3599,11 @@
           <t>workato.md</t>
         </is>
       </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>workflow-automation, integration-platform, business-process-management</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="20" t="inlineStr">
@@ -3561,6 +3656,11 @@
           <t>power-automate.md</t>
         </is>
       </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>workflow-automation, integration-platform, business-process-management</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="20" t="inlineStr">
@@ -3613,6 +3713,11 @@
           <t>ifttt.md</t>
         </is>
       </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>workflow-automation, integration-platform</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="20" t="inlineStr">
@@ -3665,6 +3770,11 @@
           <t>activepieces.md</t>
         </is>
       </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>workflow-automation, integration-platform</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="20" t="inlineStr">
@@ -3717,6 +3827,11 @@
           <t>bardeen.md</t>
         </is>
       </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>workflow-automation, sales-automation</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="20" t="inlineStr">
@@ -3769,6 +3884,11 @@
           <t>pabbly-connect.md</t>
         </is>
       </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>workflow-automation, integration-platform</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="20" t="inlineStr">
@@ -3821,6 +3941,11 @@
           <t>albato.md</t>
         </is>
       </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>workflow-automation, integration-platform</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="20" t="inlineStr">
@@ -3873,6 +3998,11 @@
           <t>integrately.md</t>
         </is>
       </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>workflow-automation, integration-platform</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="20" t="inlineStr">
@@ -3925,6 +4055,11 @@
           <t>latenode.md</t>
         </is>
       </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>workflow-automation, integration-platform</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="20" t="inlineStr">
@@ -3975,6 +4110,11 @@
       <c r="K55" t="inlineStr">
         <is>
           <t>relay-app.md</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>workflow-automation, team-collaboration</t>
         </is>
       </c>
     </row>
@@ -10622,6 +10762,11 @@
           <t>coda.md</t>
         </is>
       </c>
+      <c r="M215" t="inlineStr">
+        <is>
+          <t>document-management, database-software, no-code-platform, team-collaboration</t>
+        </is>
+      </c>
     </row>
     <row r="216" ht="25.5" customHeight="1">
       <c r="A216" s="53" t="inlineStr">
@@ -11158,6 +11303,11 @@
           <t>notion.md</t>
         </is>
       </c>
+      <c r="M228" t="inlineStr">
+        <is>
+          <t>project-management, knowledge-management, note-taking, team-collaboration, document-management, database-software</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="56" t="inlineStr">
@@ -11208,6 +11358,11 @@
       <c r="K229" t="inlineStr">
         <is>
           <t>coda.md</t>
+        </is>
+      </c>
+      <c r="M229" t="inlineStr">
+        <is>
+          <t>document-management, database-software, no-code-platform, team-collaboration</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add first 4 No-Code reviews + CRM upload script + spreadsheet update
No-Code reviews: Bubble (4.2/5), Webflow (4.4/5), Retool (4.3/5), Glide (4.0/5)
All narrative style matching ClickUp quality benchmark.
Updated spreadsheet with CRM review statuses and categories.
Added upload-batch-crm.ts for Sanity uploads.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content-templates/reviews/software_automation_tools.xlsx
+++ b/content-templates/reviews/software_automation_tools.xlsx
@@ -4748,12 +4748,22 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
           <t>High</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>hubspot-crm.md</t>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>crm-software, marketing-automation, sales-automation, email-marketing</t>
         </is>
       </c>
     </row>
@@ -4795,12 +4805,22 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
         <is>
           <t>High</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>salesforce.md</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>crm-software, sales-automation, business-process-management</t>
         </is>
       </c>
     </row>
@@ -4842,12 +4862,22 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
         <is>
           <t>High</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>pipedrive.md</t>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>crm-software, sales-automation</t>
         </is>
       </c>
     </row>
@@ -4889,12 +4919,22 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
         <is>
           <t>High</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>close.md</t>
+        </is>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>crm-software, sales-automation</t>
         </is>
       </c>
     </row>
@@ -4936,12 +4976,22 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
         <is>
           <t>High</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>apollo.md</t>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>crm-software, sales-automation, email-marketing</t>
         </is>
       </c>
     </row>
@@ -4983,12 +5033,22 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
         <is>
           <t>High</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>outreach.md</t>
+        </is>
+      </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>sales-automation</t>
         </is>
       </c>
     </row>
@@ -5030,12 +5090,22 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
         <is>
           <t>High</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>salesloft.md</t>
+        </is>
+      </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>sales-automation</t>
         </is>
       </c>
     </row>
@@ -5077,12 +5147,22 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
         <is>
           <t>High</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>lemlist.md</t>
+        </is>
+      </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>sales-automation, email-marketing</t>
         </is>
       </c>
     </row>
@@ -5124,12 +5204,22 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
         <is>
           <t>High</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>instantly.md</t>
+        </is>
+      </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>sales-automation, email-marketing</t>
         </is>
       </c>
     </row>
@@ -5171,12 +5261,22 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
         <is>
           <t>High</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>reply-io.md</t>
+        </is>
+      </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>sales-automation, email-marketing</t>
         </is>
       </c>
     </row>
@@ -5218,12 +5318,22 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
         <is>
           <t>High</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>copper.md</t>
+        </is>
+      </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>crm-software, sales-automation</t>
         </is>
       </c>
     </row>
@@ -5265,12 +5375,22 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
         <is>
           <t>High</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>zoho-crm.md</t>
+        </is>
+      </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>crm-software, sales-automation, marketing-automation</t>
         </is>
       </c>
     </row>
@@ -5312,12 +5432,22 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
         <is>
           <t>High</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>freshsales.md</t>
+        </is>
+      </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>crm-software, sales-automation</t>
         </is>
       </c>
     </row>
@@ -5359,12 +5489,22 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
         <is>
           <t>High</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>attio.md</t>
+        </is>
+      </c>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t>crm-software, sales-automation, database-software</t>
         </is>
       </c>
     </row>
@@ -5406,12 +5546,22 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
         <is>
           <t>High</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>folk.md</t>
+        </is>
+      </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>crm-software</t>
         </is>
       </c>
     </row>

</xml_diff>